<commit_message>
update sample data with region
</commit_message>
<xml_diff>
--- a/组织关系图_样例数据.xlsx
+++ b/组织关系图_样例数据.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人员清单" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="协作关系（可选）" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -446,6 +445,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -479,6 +479,11 @@
           <t>分组标签</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>区域</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -507,6 +512,11 @@
           <t>高管</t>
         </is>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>全国</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -539,6 +549,11 @@
           <t>高管</t>
         </is>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>全国</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -571,6 +586,11 @@
           <t>高管</t>
         </is>
       </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>全国</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -603,6 +623,11 @@
           <t>高管</t>
         </is>
       </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>全国</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -635,6 +660,11 @@
           <t>中层</t>
         </is>
       </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>华东</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -667,6 +697,11 @@
           <t>中层</t>
         </is>
       </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>华南</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -699,6 +734,11 @@
           <t>中层</t>
         </is>
       </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>全国</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -731,6 +771,11 @@
           <t>员工</t>
         </is>
       </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>华东</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -763,6 +808,11 @@
           <t>高管</t>
         </is>
       </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>全国</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -795,6 +845,11 @@
           <t>中层</t>
         </is>
       </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>华东</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -827,6 +882,11 @@
           <t>中层</t>
         </is>
       </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>华南</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -855,6 +915,11 @@
           <t>员工</t>
         </is>
       </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>华东</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -883,6 +948,11 @@
           <t>员工</t>
         </is>
       </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>华东</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -915,6 +985,11 @@
           <t>员工</t>
         </is>
       </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>华南</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -947,6 +1022,11 @@
           <t>中层</t>
         </is>
       </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>全国</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -975,6 +1055,11 @@
           <t>员工</t>
         </is>
       </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>华东</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1007,6 +1092,11 @@
           <t>高管</t>
         </is>
       </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>全国</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1039,6 +1129,11 @@
           <t>中层</t>
         </is>
       </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>华东</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1071,6 +1166,11 @@
           <t>员工</t>
         </is>
       </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>华南</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1103,6 +1203,11 @@
           <t>中层</t>
         </is>
       </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>全国</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1135,6 +1240,11 @@
           <t>员工</t>
         </is>
       </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>华东</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1167,6 +1277,11 @@
           <t>中层</t>
         </is>
       </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>全国</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1199,6 +1314,11 @@
           <t>员工</t>
         </is>
       </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>华东</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1231,46 +1351,9 @@
           <t>中层</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>人员A</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>人员B</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>关系类型</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>备注</t>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>全国</t>
         </is>
       </c>
     </row>

</xml_diff>